<commit_message>
Spec builder: the construction bullet wraps by measured line count, so the Korean edition's wide text is not clipped
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L3H8Na8buSZY2uPpuuSkn7
</commit_message>
<xml_diff>
--- a/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1_x3m3_KR.xlsx
+++ b/Calculation Excel Sheet/variants/Transformer_Spec_7p5to1_x3m3_KR.xlsx
@@ -127,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -141,7 +141,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -163,6 +163,9 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -576,7 +579,7 @@
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
     </row>
-    <row r="7" ht="15" customHeight="1">
+    <row r="7" ht="30" customHeight="1">
       <c r="B7" s="6" t="inlineStr">
         <is>
           <t>•   양산품 26OP-LM83W 와 같은 납작한(저배) 구조.   코어 · 보빈 · 선재 · 권선 배치는 2–4절을 만족하는 범위에서 제작사가 정하고, 전체 높이는 첫 샘플 전에 협의한다.</t>
@@ -914,12 +917,12 @@
           <t>•</t>
         </is>
       </c>
-      <c r="C31" s="6" t="inlineStr">
+      <c r="C31" s="14" t="inlineStr">
         <is>
           <t>권선 주파수</t>
         </is>
       </c>
-      <c r="E31" s="14" t="inlineStr">
+      <c r="E31" s="15" t="inlineStr">
         <is>
           <t>130 – 292 kHz</t>
         </is>
@@ -936,12 +939,12 @@
           <t>•</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="C32" s="14" t="inlineStr">
         <is>
           <t>코어 유효 단면적</t>
         </is>
       </c>
-      <c r="E32" s="14" t="inlineStr">
+      <c r="E32" s="15" t="inlineStr">
         <is>
           <t>Ae  ≥  220 mm²</t>
         </is>

</xml_diff>